<commit_message>
Deploy TWHA IG (v3對齊 Wave1+2): ConceptMap 32組, Core重構(最小上傳集)+VS-CoreUploadSet, 術語用語正名
對應原始碼 commit ffdecde。IG Publisher 建置產物(0 broken links)。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TWHealthCheckLaboratoryMap.xlsx
+++ b/TWHealthCheckLaboratoryMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="147">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-23T22:22:27+08:00</t>
+    <t>2026-07-24T13:54:16+08:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -418,6 +418,42 @@
   </si>
   <si>
     <t>18262-6</t>
+  </si>
+  <si>
+    <t>23749-5</t>
+  </si>
+  <si>
+    <t>Lead [Mass/volume] in Specimen</t>
+  </si>
+  <si>
+    <t>5671-3</t>
+  </si>
+  <si>
+    <t>Lead [Mass/volume] in Blood</t>
+  </si>
+  <si>
+    <t>56086-2</t>
+  </si>
+  <si>
+    <t>Waist Circumference</t>
+  </si>
+  <si>
+    <t>8280-0</t>
+  </si>
+  <si>
+    <t>Waist Circumference at umbilicus by Tape measure</t>
+  </si>
+  <si>
+    <t>21104-5</t>
+  </si>
+  <si>
+    <t>Pure tone audiometry - Audiometry study</t>
+  </si>
+  <si>
+    <t>89015-2</t>
+  </si>
+  <si>
+    <t>Pure tone threshold audiometry panel</t>
   </si>
 </sst>
 </file>
@@ -693,7 +729,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1223,6 +1259,57 @@
         <v>70</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="B32" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="C32" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D32" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="E32" t="s" s="2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="B33" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="C33" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="D33" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="E33" t="s" s="2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="B34" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="C34" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D34" t="s" s="2">
+        <v>145</v>
+      </c>
+      <c r="E34" t="s" s="2">
+        <v>146</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploy TWHA IG: Wave 9 錯碼移除與全面 display 語意比對
對應原始碼 commit d09500d9。移除 16 個語意錯誤代碼；324 碼完成 display 語意比對。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TWHealthCheckLaboratoryMap.xlsx
+++ b/TWHealthCheckLaboratoryMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="139">
   <si>
     <t>Property</t>
   </si>
@@ -174,18 +174,6 @@
     <t>Creatinine [Mass/volume] in Serum or Plasma</t>
   </si>
   <si>
-    <t>49154-8</t>
-  </si>
-  <si>
-    <t>Uric acid [Mass/volume] in Blood</t>
-  </si>
-  <si>
-    <t>3084-1</t>
-  </si>
-  <si>
-    <t>Uric acid [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
     <t>35200-5</t>
   </si>
   <si>
@@ -442,18 +430,6 @@
   </si>
   <si>
     <t>Waist Circumference at umbilicus by Tape measure</t>
-  </si>
-  <si>
-    <t>21104-5</t>
-  </si>
-  <si>
-    <t>Pure tone audiometry - Audiometry study</t>
-  </si>
-  <si>
-    <t>89015-2</t>
-  </si>
-  <si>
-    <t>Pure tone threshold audiometry panel</t>
   </si>
 </sst>
 </file>
@@ -729,7 +705,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -859,7 +835,7 @@
         <v>54</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s" s="2">
         <v>55</v>
@@ -876,7 +852,7 @@
         <v>58</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s" s="2">
         <v>59</v>
@@ -893,7 +869,7 @@
         <v>62</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>63</v>
@@ -910,7 +886,7 @@
         <v>66</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s" s="2">
         <v>67</v>
@@ -961,7 +937,7 @@
         <v>78</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D14" t="s" s="2">
         <v>79</v>
@@ -978,7 +954,7 @@
         <v>82</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>83</v>
@@ -995,30 +971,30 @@
         <v>86</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s" s="2">
         <v>87</v>
       </c>
       <c r="E16" t="s" s="2">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="B17" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="B17" t="s" s="2">
+      <c r="C17" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D17" t="s" s="2">
         <v>90</v>
       </c>
-      <c r="C17" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="D17" t="s" s="2">
+      <c r="E17" t="s" s="2">
         <v>91</v>
-      </c>
-      <c r="E17" t="s" s="2">
-        <v>90</v>
       </c>
     </row>
     <row r="18">
@@ -1029,7 +1005,7 @@
         <v>93</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D18" t="s" s="2">
         <v>94</v>
@@ -1063,30 +1039,30 @@
         <v>101</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D20" t="s" s="2">
         <v>102</v>
       </c>
       <c r="E20" t="s" s="2">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="B21" t="s" s="2">
         <v>104</v>
       </c>
-      <c r="B21" t="s" s="2">
+      <c r="C21" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D21" t="s" s="2">
         <v>105</v>
       </c>
-      <c r="C21" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="D21" t="s" s="2">
+      <c r="E21" t="s" s="2">
         <v>106</v>
-      </c>
-      <c r="E21" t="s" s="2">
-        <v>105</v>
       </c>
     </row>
     <row r="22">
@@ -1097,7 +1073,7 @@
         <v>108</v>
       </c>
       <c r="C22" t="s" s="2">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D22" t="s" s="2">
         <v>109</v>
@@ -1114,30 +1090,30 @@
         <v>112</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D23" t="s" s="2">
         <v>113</v>
       </c>
       <c r="E23" t="s" s="2">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="B24" t="s" s="2">
         <v>115</v>
       </c>
-      <c r="B24" t="s" s="2">
+      <c r="C24" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D24" t="s" s="2">
         <v>116</v>
       </c>
-      <c r="C24" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="D24" t="s" s="2">
+      <c r="E24" t="s" s="2">
         <v>117</v>
-      </c>
-      <c r="E24" t="s" s="2">
-        <v>116</v>
       </c>
     </row>
     <row r="25">
@@ -1168,18 +1144,18 @@
         <v>33</v>
       </c>
       <c r="D26" t="s" s="2">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="E26" t="s" s="2">
-        <v>125</v>
+        <v>95</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C27" t="s" s="2">
         <v>33</v>
@@ -1193,53 +1169,53 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="B28" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="C28" t="s" s="2">
+        <v>46</v>
+      </c>
+      <c r="D28" t="s" s="2">
+        <v>47</v>
+      </c>
+      <c r="E28" t="s" s="2">
         <v>128</v>
-      </c>
-      <c r="B28" t="s" s="2">
-        <v>129</v>
-      </c>
-      <c r="C28" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D28" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="E28" t="s" s="2">
-        <v>103</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="B29" t="s" s="2">
         <v>130</v>
       </c>
-      <c r="B29" t="s" s="2">
-        <v>131</v>
-      </c>
       <c r="C29" t="s" s="2">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="D29" t="s" s="2">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="E29" t="s" s="2">
-        <v>132</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="B30" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="C30" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D30" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="B30" t="s" s="2">
+      <c r="E30" t="s" s="2">
         <v>134</v>
-      </c>
-      <c r="C30" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D30" t="s" s="2">
-        <v>67</v>
-      </c>
-      <c r="E30" t="s" s="2">
-        <v>68</v>
       </c>
     </row>
     <row r="31">
@@ -1257,40 +1233,6 @@
       </c>
       <c r="E31" t="s" s="2">
         <v>138</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="B32" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="C32" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D32" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="E32" t="s" s="2">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s" s="2">
-        <v>143</v>
-      </c>
-      <c r="B33" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D33" t="s" s="2">
-        <v>145</v>
-      </c>
-      <c r="E33" t="s" s="2">
-        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
publish: bb554ce13737aae5fb86fdc84b4eee02239c9095 (run 30458905178)
</commit_message>
<xml_diff>
--- a/TWHealthCheckLaboratoryMap.xlsx
+++ b/TWHealthCheckLaboratoryMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="172">
   <si>
     <t>Property</t>
   </si>
@@ -421,6 +421,114 @@
   </si>
   <si>
     <t>Lead [Mass/volume] in Blood</t>
+  </si>
+  <si>
+    <t>33218-9</t>
+  </si>
+  <si>
+    <t>Bacteria [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51480-2</t>
+  </si>
+  <si>
+    <t>Bacteria [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>33219-7</t>
+  </si>
+  <si>
+    <t>Epithelial cells.squamous [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51486-9</t>
+  </si>
+  <si>
+    <t>Epithelial cells.squamous [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>33223-9</t>
+  </si>
+  <si>
+    <t>Hyaline casts [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51484-4</t>
+  </si>
+  <si>
+    <t>Hyaline casts [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>33342-7</t>
+  </si>
+  <si>
+    <t>Epithelial cells [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>87926-2</t>
+  </si>
+  <si>
+    <t>Epithelial cells [#/volume] in Urine by Automated</t>
+  </si>
+  <si>
+    <t>43755-8</t>
+  </si>
+  <si>
+    <t>Casts [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51483-6</t>
+  </si>
+  <si>
+    <t>Casts [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>46419-8</t>
+  </si>
+  <si>
+    <t>Erythrocytes [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>798-9</t>
+  </si>
+  <si>
+    <t>Erythrocytes [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>46702-7</t>
+  </si>
+  <si>
+    <t>Leukocytes [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51487-7</t>
+  </si>
+  <si>
+    <t>Leukocytes [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>50235-1</t>
+  </si>
+  <si>
+    <t>Mucus [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51478-6</t>
+  </si>
+  <si>
+    <t>Mucus [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>53324-0</t>
+  </si>
+  <si>
+    <t>Spermatozoa [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51479-4</t>
+  </si>
+  <si>
+    <t>Spermatozoa [#/volume] in Urine by Automated count</t>
   </si>
 </sst>
 </file>
@@ -696,7 +804,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1209,6 +1317,159 @@
         <v>129</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="B31" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="C31" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D31" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="E31" t="s" s="2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="B32" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="C32" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D32" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="E32" t="s" s="2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="B33" t="s" s="2">
+        <v>145</v>
+      </c>
+      <c r="C33" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D33" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="E33" t="s" s="2">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="B34" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="C34" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D34" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="E34" t="s" s="2">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="B35" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="C35" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D35" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="E35" t="s" s="2">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="B36" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="C36" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D36" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="E36" t="s" s="2">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="B37" t="s" s="2">
+        <v>161</v>
+      </c>
+      <c r="C37" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D37" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="E37" t="s" s="2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="B38" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="C38" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D38" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="E38" t="s" s="2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="2">
+        <v>168</v>
+      </c>
+      <c r="B39" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="C39" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="D39" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="E39" t="s" s="2">
+        <v>171</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
publish: 7d74192d98fae4c87b4b1ce2cebee72e690f3577 (run 30522831283)
</commit_message>
<xml_diff>
--- a/TWHealthCheckLaboratoryMap.xlsx
+++ b/TWHealthCheckLaboratoryMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="180">
   <si>
     <t>Property</t>
   </si>
@@ -529,6 +529,30 @@
   </si>
   <si>
     <t>Spermatozoa [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>3137-7</t>
+  </si>
+  <si>
+    <t>Body height Measured</t>
+  </si>
+  <si>
+    <t>8302-2</t>
+  </si>
+  <si>
+    <t>Body height</t>
+  </si>
+  <si>
+    <t>3141-9</t>
+  </si>
+  <si>
+    <t>Body weight Measured</t>
+  </si>
+  <si>
+    <t>29463-7</t>
+  </si>
+  <si>
+    <t>Body weight</t>
   </si>
 </sst>
 </file>
@@ -804,7 +828,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1470,6 +1494,40 @@
         <v>171</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="B40" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="C40" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D40" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="E40" t="s" s="2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="C41" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D41" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="E41" t="s" s="2">
+        <v>179</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
publish: f94b257771edb5bf92740e5283b87f7c0fd80dda (run 30550906663)
</commit_message>
<xml_diff>
--- a/TWHealthCheckLaboratoryMap.xlsx
+++ b/TWHealthCheckLaboratoryMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="179">
   <si>
     <t>Property</t>
   </si>
@@ -114,33 +114,30 @@
     <t>Leukocytes [#/volume] in Blood by Manual count</t>
   </si>
   <si>
+    <t>related-to</t>
+  </si>
+  <si>
+    <t>6690-2</t>
+  </si>
+  <si>
+    <t>Leukocytes [#/volume] in Blood by Automated count</t>
+  </si>
+  <si>
+    <t>26464-8</t>
+  </si>
+  <si>
+    <t>Leukocytes [#/volume] in Blood</t>
+  </si>
+  <si>
     <t>source-is-broader-than-target</t>
   </si>
   <si>
-    <t>6690-2</t>
-  </si>
-  <si>
-    <t>Leukocytes [#/volume] in Blood by Automated count</t>
-  </si>
-  <si>
-    <t>26464-8</t>
-  </si>
-  <si>
-    <t>Leukocytes [#/volume] in Blood</t>
-  </si>
-  <si>
-    <t>equivalent</t>
-  </si>
-  <si>
     <t>2888-6</t>
   </si>
   <si>
     <t>Protein [Mass/volume] in Urine</t>
   </si>
   <si>
-    <t>related-to</t>
-  </si>
-  <si>
     <t>5804-0</t>
   </si>
   <si>
@@ -153,55 +150,55 @@
     <t>Glucose [Mass/volume] in Blood</t>
   </si>
   <si>
+    <t>1558-6</t>
+  </si>
+  <si>
+    <t>Fasting glucose [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>38483-4</t>
+  </si>
+  <si>
+    <t>Creatinine [Mass/volume] in Blood</t>
+  </si>
+  <si>
+    <t>2160-0</t>
+  </si>
+  <si>
+    <t>Creatinine [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>35200-5</t>
+  </si>
+  <si>
+    <t>Cholesterol [Mass or Moles/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>2093-3</t>
+  </si>
+  <si>
+    <t>Cholesterol [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>3043-7</t>
+  </si>
+  <si>
+    <t>Triglyceride [Mass/volume] in Blood</t>
+  </si>
+  <si>
+    <t>2571-8</t>
+  </si>
+  <si>
+    <t>Triglyceride [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>13457-7</t>
+  </si>
+  <si>
+    <t>Cholesterol in LDL [Mass/volume] in Serum or Plasma by calculation</t>
+  </si>
+  <si>
     <t>source-is-narrower-than-target</t>
-  </si>
-  <si>
-    <t>1558-6</t>
-  </si>
-  <si>
-    <t>Fasting glucose [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>38483-4</t>
-  </si>
-  <si>
-    <t>Creatinine [Mass/volume] in Blood</t>
-  </si>
-  <si>
-    <t>2160-0</t>
-  </si>
-  <si>
-    <t>Creatinine [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>35200-5</t>
-  </si>
-  <si>
-    <t>Cholesterol [Mass or Moles/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>2093-3</t>
-  </si>
-  <si>
-    <t>Cholesterol [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>3043-7</t>
-  </si>
-  <si>
-    <t>Triglyceride [Mass/volume] in Blood</t>
-  </si>
-  <si>
-    <t>2571-8</t>
-  </si>
-  <si>
-    <t>Triglyceride [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>13457-7</t>
-  </si>
-  <si>
-    <t>Cholesterol in LDL [Mass/volume] in Serum or Plasma by calculation</t>
   </si>
   <si>
     <t>2089-1</t>
@@ -907,625 +904,625 @@
         <v>40</v>
       </c>
       <c r="C5" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="D5" t="s" s="2">
+      <c r="E5" t="s" s="2">
         <v>42</v>
-      </c>
-      <c r="E5" t="s" s="2">
-        <v>43</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="B6" t="s" s="2">
+      <c r="C6" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s" s="2">
         <v>45</v>
       </c>
-      <c r="C6" t="s" s="2">
+      <c r="E6" t="s" s="2">
         <v>46</v>
-      </c>
-      <c r="D6" t="s" s="2">
-        <v>47</v>
-      </c>
-      <c r="E6" t="s" s="2">
-        <v>48</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="B7" t="s" s="2">
+      <c r="E7" t="s" s="2">
         <v>50</v>
-      </c>
-      <c r="C7" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D7" t="s" s="2">
-        <v>51</v>
-      </c>
-      <c r="E7" t="s" s="2">
-        <v>52</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s" s="2">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="D8" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="B8" t="s" s="2">
+      <c r="E8" t="s" s="2">
         <v>54</v>
-      </c>
-      <c r="C8" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="D8" t="s" s="2">
-        <v>55</v>
-      </c>
-      <c r="E8" t="s" s="2">
-        <v>56</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="B9" t="s" s="2">
+      <c r="E9" t="s" s="2">
         <v>58</v>
-      </c>
-      <c r="C9" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D9" t="s" s="2">
-        <v>59</v>
-      </c>
-      <c r="E9" t="s" s="2">
-        <v>60</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s" s="2">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B10" t="s" s="2">
+      <c r="D10" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="C10" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D10" t="s" s="2">
+      <c r="E10" t="s" s="2">
         <v>63</v>
-      </c>
-      <c r="E10" t="s" s="2">
-        <v>64</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="B11" t="s" s="2">
+      <c r="C11" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D11" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="C11" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D11" t="s" s="2">
+      <c r="E11" t="s" s="2">
         <v>67</v>
-      </c>
-      <c r="E11" t="s" s="2">
-        <v>68</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
+        <v>68</v>
+      </c>
+      <c r="B12" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="B12" t="s" s="2">
+      <c r="C12" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="C12" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D12" t="s" s="2">
+      <c r="E12" t="s" s="2">
         <v>71</v>
-      </c>
-      <c r="E12" t="s" s="2">
-        <v>72</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
+        <v>72</v>
+      </c>
+      <c r="B13" t="s" s="2">
         <v>73</v>
       </c>
-      <c r="B13" t="s" s="2">
+      <c r="C13" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s" s="2">
         <v>74</v>
       </c>
-      <c r="C13" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D13" t="s" s="2">
+      <c r="E13" t="s" s="2">
         <v>75</v>
-      </c>
-      <c r="E13" t="s" s="2">
-        <v>76</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="B14" t="s" s="2">
+      <c r="C14" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="D14" t="s" s="2">
         <v>78</v>
       </c>
-      <c r="C14" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D14" t="s" s="2">
+      <c r="E14" t="s" s="2">
         <v>79</v>
-      </c>
-      <c r="E14" t="s" s="2">
-        <v>80</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="B15" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="B15" t="s" s="2">
+      <c r="C15" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D15" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="C15" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D15" t="s" s="2">
+      <c r="E15" t="s" s="2">
         <v>83</v>
-      </c>
-      <c r="E15" t="s" s="2">
-        <v>84</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="B16" t="s" s="2">
         <v>85</v>
-      </c>
-      <c r="B16" t="s" s="2">
-        <v>86</v>
       </c>
       <c r="C16" t="s" s="2">
         <v>38</v>
       </c>
       <c r="D16" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="E16" t="s" s="2">
         <v>87</v>
-      </c>
-      <c r="E16" t="s" s="2">
-        <v>88</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="B17" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="B17" t="s" s="2">
+      <c r="C17" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s" s="2">
         <v>90</v>
       </c>
-      <c r="C17" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D17" t="s" s="2">
+      <c r="E17" t="s" s="2">
         <v>91</v>
-      </c>
-      <c r="E17" t="s" s="2">
-        <v>92</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="B18" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="B18" t="s" s="2">
+      <c r="C18" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="D18" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="C18" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D18" t="s" s="2">
+      <c r="E18" t="s" s="2">
         <v>95</v>
-      </c>
-      <c r="E18" t="s" s="2">
-        <v>96</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="B19" t="s" s="2">
         <v>97</v>
       </c>
-      <c r="B19" t="s" s="2">
+      <c r="C19" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="D19" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="C19" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D19" t="s" s="2">
+      <c r="E19" t="s" s="2">
         <v>99</v>
-      </c>
-      <c r="E19" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="B20" t="s" s="2">
         <v>101</v>
       </c>
-      <c r="B20" t="s" s="2">
+      <c r="C20" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D20" t="s" s="2">
         <v>102</v>
       </c>
-      <c r="C20" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D20" t="s" s="2">
+      <c r="E20" t="s" s="2">
         <v>103</v>
-      </c>
-      <c r="E20" t="s" s="2">
-        <v>104</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="B21" t="s" s="2">
         <v>105</v>
       </c>
-      <c r="B21" t="s" s="2">
+      <c r="C21" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="D21" t="s" s="2">
         <v>106</v>
       </c>
-      <c r="C21" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D21" t="s" s="2">
+      <c r="E21" t="s" s="2">
         <v>107</v>
-      </c>
-      <c r="E21" t="s" s="2">
-        <v>108</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="B22" t="s" s="2">
         <v>109</v>
       </c>
-      <c r="B22" t="s" s="2">
+      <c r="C22" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="D22" t="s" s="2">
         <v>110</v>
       </c>
-      <c r="C22" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D22" t="s" s="2">
+      <c r="E22" t="s" s="2">
         <v>111</v>
-      </c>
-      <c r="E22" t="s" s="2">
-        <v>112</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="B23" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="B23" t="s" s="2">
+      <c r="C23" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="D23" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="C23" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D23" t="s" s="2">
+      <c r="E23" t="s" s="2">
         <v>115</v>
-      </c>
-      <c r="E23" t="s" s="2">
-        <v>116</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="B24" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="B24" t="s" s="2">
-        <v>118</v>
-      </c>
       <c r="C24" t="s" s="2">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="D24" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="E24" t="s" s="2">
         <v>95</v>
-      </c>
-      <c r="E24" t="s" s="2">
-        <v>96</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="B25" t="s" s="2">
         <v>119</v>
       </c>
-      <c r="B25" t="s" s="2">
-        <v>120</v>
-      </c>
       <c r="C25" t="s" s="2">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="E25" t="s" s="2">
         <v>99</v>
-      </c>
-      <c r="E25" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="B26" t="s" s="2">
         <v>121</v>
       </c>
-      <c r="B26" t="s" s="2">
+      <c r="C26" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="D26" t="s" s="2">
+        <v>45</v>
+      </c>
+      <c r="E26" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="C26" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="D26" t="s" s="2">
-        <v>47</v>
-      </c>
-      <c r="E26" t="s" s="2">
-        <v>123</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="B27" t="s" s="2">
         <v>124</v>
       </c>
-      <c r="B27" t="s" s="2">
-        <v>125</v>
-      </c>
       <c r="C27" t="s" s="2">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s" s="2">
+        <v>62</v>
+      </c>
+      <c r="E27" t="s" s="2">
         <v>63</v>
-      </c>
-      <c r="E27" t="s" s="2">
-        <v>64</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="B28" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="B28" t="s" s="2">
+      <c r="C28" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D28" t="s" s="2">
         <v>127</v>
       </c>
-      <c r="C28" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D28" t="s" s="2">
+      <c r="E28" t="s" s="2">
         <v>128</v>
-      </c>
-      <c r="E28" t="s" s="2">
-        <v>129</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="B29" t="s" s="2">
         <v>130</v>
       </c>
-      <c r="B29" t="s" s="2">
+      <c r="C29" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D29" t="s" s="2">
         <v>131</v>
       </c>
-      <c r="C29" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D29" t="s" s="2">
+      <c r="E29" t="s" s="2">
         <v>132</v>
-      </c>
-      <c r="E29" t="s" s="2">
-        <v>133</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="B30" t="s" s="2">
         <v>134</v>
       </c>
-      <c r="B30" t="s" s="2">
-        <v>135</v>
-      </c>
       <c r="C30" t="s" s="2">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D30" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="E30" t="s" s="2">
         <v>128</v>
-      </c>
-      <c r="E30" t="s" s="2">
-        <v>129</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="B31" t="s" s="2">
         <v>136</v>
       </c>
-      <c r="B31" t="s" s="2">
+      <c r="C31" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D31" t="s" s="2">
         <v>137</v>
       </c>
-      <c r="C31" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D31" t="s" s="2">
+      <c r="E31" t="s" s="2">
         <v>138</v>
-      </c>
-      <c r="E31" t="s" s="2">
-        <v>139</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="B32" t="s" s="2">
         <v>140</v>
       </c>
-      <c r="B32" t="s" s="2">
+      <c r="C32" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D32" t="s" s="2">
         <v>141</v>
       </c>
-      <c r="C32" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D32" t="s" s="2">
+      <c r="E32" t="s" s="2">
         <v>142</v>
-      </c>
-      <c r="E32" t="s" s="2">
-        <v>143</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="B33" t="s" s="2">
         <v>144</v>
       </c>
-      <c r="B33" t="s" s="2">
+      <c r="C33" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D33" t="s" s="2">
         <v>145</v>
       </c>
-      <c r="C33" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D33" t="s" s="2">
+      <c r="E33" t="s" s="2">
         <v>146</v>
-      </c>
-      <c r="E33" t="s" s="2">
-        <v>147</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="B34" t="s" s="2">
         <v>148</v>
       </c>
-      <c r="B34" t="s" s="2">
+      <c r="C34" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D34" t="s" s="2">
         <v>149</v>
       </c>
-      <c r="C34" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D34" t="s" s="2">
+      <c r="E34" t="s" s="2">
         <v>150</v>
-      </c>
-      <c r="E34" t="s" s="2">
-        <v>151</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="B35" t="s" s="2">
         <v>152</v>
       </c>
-      <c r="B35" t="s" s="2">
+      <c r="C35" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D35" t="s" s="2">
         <v>153</v>
       </c>
-      <c r="C35" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D35" t="s" s="2">
+      <c r="E35" t="s" s="2">
         <v>154</v>
-      </c>
-      <c r="E35" t="s" s="2">
-        <v>155</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="B36" t="s" s="2">
         <v>156</v>
       </c>
-      <c r="B36" t="s" s="2">
+      <c r="C36" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D36" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="C36" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D36" t="s" s="2">
+      <c r="E36" t="s" s="2">
         <v>158</v>
-      </c>
-      <c r="E36" t="s" s="2">
-        <v>159</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="B37" t="s" s="2">
         <v>160</v>
       </c>
-      <c r="B37" t="s" s="2">
+      <c r="C37" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D37" t="s" s="2">
         <v>161</v>
       </c>
-      <c r="C37" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D37" t="s" s="2">
+      <c r="E37" t="s" s="2">
         <v>162</v>
-      </c>
-      <c r="E37" t="s" s="2">
-        <v>163</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="B38" t="s" s="2">
         <v>164</v>
       </c>
-      <c r="B38" t="s" s="2">
+      <c r="C38" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D38" t="s" s="2">
         <v>165</v>
       </c>
-      <c r="C38" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D38" t="s" s="2">
+      <c r="E38" t="s" s="2">
         <v>166</v>
-      </c>
-      <c r="E38" t="s" s="2">
-        <v>167</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
+        <v>167</v>
+      </c>
+      <c r="B39" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="B39" t="s" s="2">
+      <c r="C39" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D39" t="s" s="2">
         <v>169</v>
       </c>
-      <c r="C39" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="D39" t="s" s="2">
+      <c r="E39" t="s" s="2">
         <v>170</v>
-      </c>
-      <c r="E39" t="s" s="2">
-        <v>171</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
+        <v>171</v>
+      </c>
+      <c r="B40" t="s" s="2">
         <v>172</v>
       </c>
-      <c r="B40" t="s" s="2">
+      <c r="C40" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="D40" t="s" s="2">
         <v>173</v>
       </c>
-      <c r="C40" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D40" t="s" s="2">
+      <c r="E40" t="s" s="2">
         <v>174</v>
-      </c>
-      <c r="E40" t="s" s="2">
-        <v>175</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="B41" t="s" s="2">
         <v>176</v>
       </c>
-      <c r="B41" t="s" s="2">
+      <c r="C41" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="D41" t="s" s="2">
         <v>177</v>
       </c>
-      <c r="C41" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D41" t="s" s="2">
+      <c r="E41" t="s" s="2">
         <v>178</v>
-      </c>
-      <c r="E41" t="s" s="2">
-        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
publish: feff6d76ceb85164daa2237f6b6718d314ce7cf4 (run 30553278310)
</commit_message>
<xml_diff>
--- a/TWHealthCheckLaboratoryMap.xlsx
+++ b/TWHealthCheckLaboratoryMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="185">
   <si>
     <t>Property</t>
   </si>
@@ -132,10 +132,418 @@
     <t>source-is-broader-than-target</t>
   </si>
   <si>
-    <t>2888-6</t>
-  </si>
-  <si>
-    <t>Protein [Mass/volume] in Urine</t>
+    <t>2339-0</t>
+  </si>
+  <si>
+    <t>Glucose [Mass/volume] in Blood</t>
+  </si>
+  <si>
+    <t>1558-6</t>
+  </si>
+  <si>
+    <t>Fasting glucose [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>38483-4</t>
+  </si>
+  <si>
+    <t>Creatinine [Mass/volume] in Blood</t>
+  </si>
+  <si>
+    <t>2160-0</t>
+  </si>
+  <si>
+    <t>Creatinine [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>35200-5</t>
+  </si>
+  <si>
+    <t>Cholesterol [Mass or Moles/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>2093-3</t>
+  </si>
+  <si>
+    <t>Cholesterol [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>3043-7</t>
+  </si>
+  <si>
+    <t>Triglyceride [Mass/volume] in Blood</t>
+  </si>
+  <si>
+    <t>2571-8</t>
+  </si>
+  <si>
+    <t>Triglyceride [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>13457-7</t>
+  </si>
+  <si>
+    <t>Cholesterol in LDL [Mass/volume] in Serum or Plasma by calculation</t>
+  </si>
+  <si>
+    <t>source-is-narrower-than-target</t>
+  </si>
+  <si>
+    <t>2089-1</t>
+  </si>
+  <si>
+    <t>Cholesterol in LDL [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>33914-3</t>
+  </si>
+  <si>
+    <t>Glomerular filtration rate [Volume Rate/Area] in Serum or Plasma by Creatinine-based formula (MDRD)/1.73 sq M</t>
+  </si>
+  <si>
+    <t>98979-8</t>
+  </si>
+  <si>
+    <t>Glomerular filtration rate [Volume Rate/Area] in Serum, Plasma or Blood by Creatinine-based formula (CKD-EPI 2021)/1.73 sq M</t>
+  </si>
+  <si>
+    <t>5195-3</t>
+  </si>
+  <si>
+    <t>Hepatitis B virus surface Ag [Presence] in Serum</t>
+  </si>
+  <si>
+    <t>5196-1</t>
+  </si>
+  <si>
+    <t>Hepatitis B virus surface Ag [Presence] in Serum or Plasma by Immunoassay</t>
+  </si>
+  <si>
+    <t>16128-1</t>
+  </si>
+  <si>
+    <t>Hepatitis C virus Ab [Presence] in Serum</t>
+  </si>
+  <si>
+    <t>13955-0</t>
+  </si>
+  <si>
+    <t>Hepatitis C virus Ab [Presence] in Serum or Plasma by Immunoassay</t>
+  </si>
+  <si>
+    <t>26515-7</t>
+  </si>
+  <si>
+    <t>Platelets [#/volume] in Blood</t>
+  </si>
+  <si>
+    <t>777-3</t>
+  </si>
+  <si>
+    <t>Platelets [#/volume] in Blood by Automated count</t>
+  </si>
+  <si>
+    <t>30428-7</t>
+  </si>
+  <si>
+    <t>MCV [Entitic mean volume] in Red Blood Cells</t>
+  </si>
+  <si>
+    <t>787-2</t>
+  </si>
+  <si>
+    <t>MCV [Entitic mean volume] in Red Blood Cells by Automated count</t>
+  </si>
+  <si>
+    <t>28539-5</t>
+  </si>
+  <si>
+    <t>MCH [Entitic mass]</t>
+  </si>
+  <si>
+    <t>785-6</t>
+  </si>
+  <si>
+    <t>MCH [Entitic mass] by Automated count</t>
+  </si>
+  <si>
+    <t>26508-2</t>
+  </si>
+  <si>
+    <t>Neutrophils/100 leukocytes in Blood by Manual count</t>
+  </si>
+  <si>
+    <t>770-8</t>
+  </si>
+  <si>
+    <t>Neutrophils/Leukocytes in Blood by Automated count</t>
+  </si>
+  <si>
+    <t>30239-8</t>
+  </si>
+  <si>
+    <t>Aspartate aminotransferase [Enzymatic activity/volume] in Serum or Plasma by With P-5'-P</t>
+  </si>
+  <si>
+    <t>1920-8</t>
+  </si>
+  <si>
+    <t>Aspartate aminotransferase [Enzymatic activity/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>1743-4</t>
+  </si>
+  <si>
+    <t>Alanine aminotransferase [Enzymatic activity/volume] in Serum or Plasma by With P-5'-P</t>
+  </si>
+  <si>
+    <t>1742-6</t>
+  </si>
+  <si>
+    <t>Alanine aminotransferase [Enzymatic activity/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>59261-8</t>
+  </si>
+  <si>
+    <t>Hemoglobin A1c/Hemoglobin.total standardized per IFCC-RMP for CDT in Blood</t>
+  </si>
+  <si>
+    <t>4548-4</t>
+  </si>
+  <si>
+    <t>Hemoglobin A1c/Hemoglobin.total in Blood</t>
+  </si>
+  <si>
+    <t>3016-3</t>
+  </si>
+  <si>
+    <t>Thyrotropin [Units/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>11580-8</t>
+  </si>
+  <si>
+    <t>Thyrotropin [Units/volume] in Serum or Plasma by Detection limit &lt;= 0.005 mIU/L</t>
+  </si>
+  <si>
+    <t>83082-8</t>
+  </si>
+  <si>
+    <t>Cancer Ag 125 [Units/volume] in Serum or Plasma by Immunoassay</t>
+  </si>
+  <si>
+    <t>10334-1</t>
+  </si>
+  <si>
+    <t>Cancer Ag 125 [Units/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>83085-1</t>
+  </si>
+  <si>
+    <t>Carcinoembryonic Ag [Mass/volume] in Serum or Plasma by Immunoassay</t>
+  </si>
+  <si>
+    <t>2039-6</t>
+  </si>
+  <si>
+    <t>Carcinoembryonic Ag [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>88112-8</t>
+  </si>
+  <si>
+    <t>Aspartate aminotransferase [Enzymatic activity/volume] in Serum or Plasma by No addition of P-5'-P</t>
+  </si>
+  <si>
+    <t>1744-2</t>
+  </si>
+  <si>
+    <t>Alanine aminotransferase [Enzymatic activity/volume] in Serum or Plasma by No addition of P-5'-P</t>
+  </si>
+  <si>
+    <t>2345-7</t>
+  </si>
+  <si>
+    <t>Glucose [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>Fasting Glucose [Mass/volume] in Serum or Plasma</t>
+  </si>
+  <si>
+    <t>18262-6</t>
+  </si>
+  <si>
+    <t>Cholesterol in LDL [Mass/volume] in Serum or Plasma by Direct assay</t>
+  </si>
+  <si>
+    <t>23749-5</t>
+  </si>
+  <si>
+    <t>Lead [Mass/volume] in Specimen</t>
+  </si>
+  <si>
+    <t>77307-7</t>
+  </si>
+  <si>
+    <t>Lead [Mass/volume] in Venous blood</t>
+  </si>
+  <si>
+    <t>56086-2</t>
+  </si>
+  <si>
+    <t>Waist Circumference</t>
+  </si>
+  <si>
+    <t>8280-0</t>
+  </si>
+  <si>
+    <t>Waist Circumference at umbilicus by Tape measure</t>
+  </si>
+  <si>
+    <t>5671-3</t>
+  </si>
+  <si>
+    <t>Lead [Mass/volume] in Blood</t>
+  </si>
+  <si>
+    <t>33218-9</t>
+  </si>
+  <si>
+    <t>Bacteria [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51480-2</t>
+  </si>
+  <si>
+    <t>Bacteria [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>33219-7</t>
+  </si>
+  <si>
+    <t>Epithelial cells.squamous [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51486-9</t>
+  </si>
+  <si>
+    <t>Epithelial cells.squamous [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>33223-9</t>
+  </si>
+  <si>
+    <t>Hyaline casts [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51484-4</t>
+  </si>
+  <si>
+    <t>Hyaline casts [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>33342-7</t>
+  </si>
+  <si>
+    <t>Epithelial cells [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>87926-2</t>
+  </si>
+  <si>
+    <t>Epithelial cells [#/volume] in Urine by Automated</t>
+  </si>
+  <si>
+    <t>43755-8</t>
+  </si>
+  <si>
+    <t>Casts [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51483-6</t>
+  </si>
+  <si>
+    <t>Casts [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>46419-8</t>
+  </si>
+  <si>
+    <t>Erythrocytes [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>798-9</t>
+  </si>
+  <si>
+    <t>Erythrocytes [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>46702-7</t>
+  </si>
+  <si>
+    <t>Leukocytes [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51487-7</t>
+  </si>
+  <si>
+    <t>Leukocytes [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>50235-1</t>
+  </si>
+  <si>
+    <t>Mucus [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51478-6</t>
+  </si>
+  <si>
+    <t>Mucus [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>53324-0</t>
+  </si>
+  <si>
+    <t>Spermatozoa [#/area] in Urine sediment by Automated count</t>
+  </si>
+  <si>
+    <t>51479-4</t>
+  </si>
+  <si>
+    <t>Spermatozoa [#/volume] in Urine by Automated count</t>
+  </si>
+  <si>
+    <t>3137-7</t>
+  </si>
+  <si>
+    <t>Body height Measured</t>
+  </si>
+  <si>
+    <t>8302-2</t>
+  </si>
+  <si>
+    <t>Body height</t>
+  </si>
+  <si>
+    <t>3141-9</t>
+  </si>
+  <si>
+    <t>Body weight Measured</t>
+  </si>
+  <si>
+    <t>29463-7</t>
+  </si>
+  <si>
+    <t>Body weight</t>
+  </si>
+  <si>
+    <t>57735-3</t>
+  </si>
+  <si>
+    <t>Protein [Presence] in Urine by Automated test strip</t>
   </si>
   <si>
     <t>5804-0</t>
@@ -144,412 +552,22 @@
     <t>Protein [Mass/volume] in Urine by Test strip</t>
   </si>
   <si>
-    <t>2339-0</t>
-  </si>
-  <si>
-    <t>Glucose [Mass/volume] in Blood</t>
-  </si>
-  <si>
-    <t>1558-6</t>
-  </si>
-  <si>
-    <t>Fasting glucose [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>38483-4</t>
-  </si>
-  <si>
-    <t>Creatinine [Mass/volume] in Blood</t>
-  </si>
-  <si>
-    <t>2160-0</t>
-  </si>
-  <si>
-    <t>Creatinine [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>35200-5</t>
-  </si>
-  <si>
-    <t>Cholesterol [Mass or Moles/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>2093-3</t>
-  </si>
-  <si>
-    <t>Cholesterol [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>3043-7</t>
-  </si>
-  <si>
-    <t>Triglyceride [Mass/volume] in Blood</t>
-  </si>
-  <si>
-    <t>2571-8</t>
-  </si>
-  <si>
-    <t>Triglyceride [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>13457-7</t>
-  </si>
-  <si>
-    <t>Cholesterol in LDL [Mass/volume] in Serum or Plasma by calculation</t>
-  </si>
-  <si>
-    <t>source-is-narrower-than-target</t>
-  </si>
-  <si>
-    <t>2089-1</t>
-  </si>
-  <si>
-    <t>Cholesterol in LDL [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>33914-3</t>
-  </si>
-  <si>
-    <t>Glomerular filtration rate [Volume Rate/Area] in Serum or Plasma by Creatinine-based formula (MDRD)/1.73 sq M</t>
-  </si>
-  <si>
-    <t>98979-8</t>
-  </si>
-  <si>
-    <t>Glomerular filtration rate [Volume Rate/Area] in Serum, Plasma or Blood by Creatinine-based formula (CKD-EPI 2021)/1.73 sq M</t>
-  </si>
-  <si>
-    <t>5195-3</t>
-  </si>
-  <si>
-    <t>Hepatitis B virus surface Ag [Presence] in Serum</t>
-  </si>
-  <si>
-    <t>5196-1</t>
-  </si>
-  <si>
-    <t>Hepatitis B virus surface Ag [Presence] in Serum or Plasma by Immunoassay</t>
-  </si>
-  <si>
-    <t>16128-1</t>
-  </si>
-  <si>
-    <t>Hepatitis C virus Ab [Presence] in Serum</t>
-  </si>
-  <si>
-    <t>13955-0</t>
-  </si>
-  <si>
-    <t>Hepatitis C virus Ab [Presence] in Serum or Plasma by Immunoassay</t>
-  </si>
-  <si>
-    <t>26515-7</t>
-  </si>
-  <si>
-    <t>Platelets [#/volume] in Blood</t>
-  </si>
-  <si>
-    <t>777-3</t>
-  </si>
-  <si>
-    <t>Platelets [#/volume] in Blood by Automated count</t>
-  </si>
-  <si>
-    <t>30428-7</t>
-  </si>
-  <si>
-    <t>MCV [Entitic mean volume] in Red Blood Cells</t>
-  </si>
-  <si>
-    <t>787-2</t>
-  </si>
-  <si>
-    <t>MCV [Entitic mean volume] in Red Blood Cells by Automated count</t>
-  </si>
-  <si>
-    <t>28539-5</t>
-  </si>
-  <si>
-    <t>MCH [Entitic mass]</t>
-  </si>
-  <si>
-    <t>785-6</t>
-  </si>
-  <si>
-    <t>MCH [Entitic mass] by Automated count</t>
-  </si>
-  <si>
-    <t>26508-2</t>
-  </si>
-  <si>
-    <t>Neutrophils/100 leukocytes in Blood by Manual count</t>
-  </si>
-  <si>
-    <t>770-8</t>
-  </si>
-  <si>
-    <t>Neutrophils/Leukocytes in Blood by Automated count</t>
-  </si>
-  <si>
-    <t>30239-8</t>
-  </si>
-  <si>
-    <t>Aspartate aminotransferase [Enzymatic activity/volume] in Serum or Plasma by With P-5'-P</t>
-  </si>
-  <si>
-    <t>1920-8</t>
-  </si>
-  <si>
-    <t>Aspartate aminotransferase [Enzymatic activity/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>1743-4</t>
-  </si>
-  <si>
-    <t>Alanine aminotransferase [Enzymatic activity/volume] in Serum or Plasma by With P-5'-P</t>
-  </si>
-  <si>
-    <t>1742-6</t>
-  </si>
-  <si>
-    <t>Alanine aminotransferase [Enzymatic activity/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>59261-8</t>
-  </si>
-  <si>
-    <t>Hemoglobin A1c/Hemoglobin.total standardized per IFCC-RMP for CDT in Blood</t>
-  </si>
-  <si>
-    <t>4548-4</t>
-  </si>
-  <si>
-    <t>Hemoglobin A1c/Hemoglobin.total in Blood</t>
-  </si>
-  <si>
-    <t>3016-3</t>
-  </si>
-  <si>
-    <t>Thyrotropin [Units/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>11580-8</t>
-  </si>
-  <si>
-    <t>Thyrotropin [Units/volume] in Serum or Plasma by Detection limit &lt;= 0.005 mIU/L</t>
-  </si>
-  <si>
-    <t>83082-8</t>
-  </si>
-  <si>
-    <t>Cancer Ag 125 [Units/volume] in Serum or Plasma by Immunoassay</t>
-  </si>
-  <si>
-    <t>10334-1</t>
-  </si>
-  <si>
-    <t>Cancer Ag 125 [Units/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>83085-1</t>
-  </si>
-  <si>
-    <t>Carcinoembryonic Ag [Mass/volume] in Serum or Plasma by Immunoassay</t>
-  </si>
-  <si>
-    <t>2039-6</t>
-  </si>
-  <si>
-    <t>Carcinoembryonic Ag [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>88112-8</t>
-  </si>
-  <si>
-    <t>Aspartate aminotransferase [Enzymatic activity/volume] in Serum or Plasma by No addition of P-5'-P</t>
-  </si>
-  <si>
-    <t>1744-2</t>
-  </si>
-  <si>
-    <t>Alanine aminotransferase [Enzymatic activity/volume] in Serum or Plasma by No addition of P-5'-P</t>
-  </si>
-  <si>
-    <t>2345-7</t>
-  </si>
-  <si>
-    <t>Glucose [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>Fasting Glucose [Mass/volume] in Serum or Plasma</t>
-  </si>
-  <si>
-    <t>18262-6</t>
-  </si>
-  <si>
-    <t>Cholesterol in LDL [Mass/volume] in Serum or Plasma by Direct assay</t>
-  </si>
-  <si>
-    <t>23749-5</t>
-  </si>
-  <si>
-    <t>Lead [Mass/volume] in Specimen</t>
-  </si>
-  <si>
-    <t>77307-7</t>
-  </si>
-  <si>
-    <t>Lead [Mass/volume] in Venous blood</t>
-  </si>
-  <si>
-    <t>56086-2</t>
-  </si>
-  <si>
-    <t>Waist Circumference</t>
-  </si>
-  <si>
-    <t>8280-0</t>
-  </si>
-  <si>
-    <t>Waist Circumference at umbilicus by Tape measure</t>
-  </si>
-  <si>
-    <t>5671-3</t>
-  </si>
-  <si>
-    <t>Lead [Mass/volume] in Blood</t>
-  </si>
-  <si>
-    <t>33218-9</t>
-  </si>
-  <si>
-    <t>Bacteria [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>51480-2</t>
-  </si>
-  <si>
-    <t>Bacteria [#/volume] in Urine by Automated count</t>
-  </si>
-  <si>
-    <t>33219-7</t>
-  </si>
-  <si>
-    <t>Epithelial cells.squamous [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>51486-9</t>
-  </si>
-  <si>
-    <t>Epithelial cells.squamous [#/volume] in Urine by Automated count</t>
-  </si>
-  <si>
-    <t>33223-9</t>
-  </si>
-  <si>
-    <t>Hyaline casts [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>51484-4</t>
-  </si>
-  <si>
-    <t>Hyaline casts [#/volume] in Urine by Automated count</t>
-  </si>
-  <si>
-    <t>33342-7</t>
-  </si>
-  <si>
-    <t>Epithelial cells [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>87926-2</t>
-  </si>
-  <si>
-    <t>Epithelial cells [#/volume] in Urine by Automated</t>
-  </si>
-  <si>
-    <t>43755-8</t>
-  </si>
-  <si>
-    <t>Casts [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>51483-6</t>
-  </si>
-  <si>
-    <t>Casts [#/volume] in Urine by Automated count</t>
-  </si>
-  <si>
-    <t>46419-8</t>
-  </si>
-  <si>
-    <t>Erythrocytes [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>798-9</t>
-  </si>
-  <si>
-    <t>Erythrocytes [#/volume] in Urine by Automated count</t>
-  </si>
-  <si>
-    <t>46702-7</t>
-  </si>
-  <si>
-    <t>Leukocytes [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>51487-7</t>
-  </si>
-  <si>
-    <t>Leukocytes [#/volume] in Urine by Automated count</t>
-  </si>
-  <si>
-    <t>50235-1</t>
-  </si>
-  <si>
-    <t>Mucus [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>51478-6</t>
-  </si>
-  <si>
-    <t>Mucus [#/volume] in Urine by Automated count</t>
-  </si>
-  <si>
-    <t>53324-0</t>
-  </si>
-  <si>
-    <t>Spermatozoa [#/area] in Urine sediment by Automated count</t>
-  </si>
-  <si>
-    <t>51479-4</t>
-  </si>
-  <si>
-    <t>Spermatozoa [#/volume] in Urine by Automated count</t>
-  </si>
-  <si>
-    <t>3137-7</t>
-  </si>
-  <si>
-    <t>Body height Measured</t>
-  </si>
-  <si>
-    <t>8302-2</t>
-  </si>
-  <si>
-    <t>Body height</t>
-  </si>
-  <si>
-    <t>3141-9</t>
-  </si>
-  <si>
-    <t>Body weight Measured</t>
-  </si>
-  <si>
-    <t>29463-7</t>
-  </si>
-  <si>
-    <t>Body weight</t>
+    <t>63557-3</t>
+  </si>
+  <si>
+    <t>Hepatitis B virus surface Ag [Units/volume] in Serum or Plasma by Immunoassay</t>
+  </si>
+  <si>
+    <t>19876-2</t>
+  </si>
+  <si>
+    <t>Forced vital capacity [Volume] Respiratory system by Spirometry --pre bronchodilation</t>
+  </si>
+  <si>
+    <t>19868-9</t>
+  </si>
+  <si>
+    <t>Forced vital capacity [Volume] Respiratory system by Spirometry</t>
   </si>
 </sst>
 </file>
@@ -825,7 +843,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -938,7 +956,7 @@
         <v>48</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s" s="2">
         <v>49</v>
@@ -955,7 +973,7 @@
         <v>52</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s" s="2">
         <v>53</v>
@@ -972,24 +990,24 @@
         <v>56</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>62</v>
@@ -1040,7 +1058,7 @@
         <v>73</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D13" t="s" s="2">
         <v>74</v>
@@ -1057,7 +1075,7 @@
         <v>77</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D14" t="s" s="2">
         <v>78</v>
@@ -1074,7 +1092,7 @@
         <v>81</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>82</v>
@@ -1091,7 +1109,7 @@
         <v>85</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D16" t="s" s="2">
         <v>86</v>
@@ -1108,7 +1126,7 @@
         <v>89</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s" s="2">
         <v>90</v>
@@ -1125,7 +1143,7 @@
         <v>93</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D18" t="s" s="2">
         <v>94</v>
@@ -1142,7 +1160,7 @@
         <v>97</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="D19" t="s" s="2">
         <v>98</v>
@@ -1159,7 +1177,7 @@
         <v>101</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D20" t="s" s="2">
         <v>102</v>
@@ -1176,7 +1194,7 @@
         <v>105</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="D21" t="s" s="2">
         <v>106</v>
@@ -1193,7 +1211,7 @@
         <v>109</v>
       </c>
       <c r="C22" t="s" s="2">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D22" t="s" s="2">
         <v>110</v>
@@ -1210,24 +1228,24 @@
         <v>113</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D23" t="s" s="2">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="E23" t="s" s="2">
-        <v>115</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C24" t="s" s="2">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D24" t="s" s="2">
         <v>94</v>
@@ -1238,53 +1256,53 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="B25" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="C25" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="D25" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="E25" t="s" s="2">
         <v>118</v>
-      </c>
-      <c r="B25" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="C25" t="s" s="2">
-        <v>61</v>
-      </c>
-      <c r="D25" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="E25" t="s" s="2">
-        <v>99</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="B26" t="s" s="2">
         <v>120</v>
       </c>
-      <c r="B26" t="s" s="2">
-        <v>121</v>
-      </c>
       <c r="C26" t="s" s="2">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="D26" t="s" s="2">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="E26" t="s" s="2">
-        <v>122</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="B27" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="C27" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D27" t="s" s="2">
         <v>123</v>
       </c>
-      <c r="B27" t="s" s="2">
+      <c r="E27" t="s" s="2">
         <v>124</v>
-      </c>
-      <c r="C27" t="s" s="2">
-        <v>61</v>
-      </c>
-      <c r="D27" t="s" s="2">
-        <v>62</v>
-      </c>
-      <c r="E27" t="s" s="2">
-        <v>63</v>
       </c>
     </row>
     <row r="28">
@@ -1315,27 +1333,27 @@
         <v>33</v>
       </c>
       <c r="D29" t="s" s="2">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="E29" t="s" s="2">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="B30" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="C30" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D30" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="B30" t="s" s="2">
+      <c r="E30" t="s" s="2">
         <v>134</v>
-      </c>
-      <c r="C30" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="D30" t="s" s="2">
-        <v>127</v>
-      </c>
-      <c r="E30" t="s" s="2">
-        <v>128</v>
       </c>
     </row>
     <row r="31">
@@ -1482,7 +1500,7 @@
         <v>168</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="D39" t="s" s="2">
         <v>169</v>
@@ -1499,7 +1517,7 @@
         <v>172</v>
       </c>
       <c r="C40" t="s" s="2">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D40" t="s" s="2">
         <v>173</v>
@@ -1516,13 +1534,47 @@
         <v>176</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D41" t="s" s="2">
         <v>177</v>
       </c>
       <c r="E41" t="s" s="2">
         <v>178</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="B42" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="C42" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="D42" t="s" s="2">
+        <v>66</v>
+      </c>
+      <c r="E42" t="s" s="2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="B43" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="C43" t="s" s="2">
+        <v>57</v>
+      </c>
+      <c r="D43" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="E43" t="s" s="2">
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>